<commit_message>
updated the test kit so it has proper run files
</commit_message>
<xml_diff>
--- a/TestKit/TestKit/Q1/Environment.xlsx
+++ b/TestKit/TestKit/Q1/Environment.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\School\NET\Recorder_NetWorking\WpfUI\Resources\Templates\DotnetNetworking\Question\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\School\NET\NewQ\Testkit\NpCap\Q1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1734F499-C41A-4E64-ABE7-48FF16AEE5D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0924FCFF-8A3F-48B4-AEB9-A244B8EFAB04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
     <sheet name="Action" sheetId="3" r:id="rId2"/>
-    <sheet name="Run" sheetId="4" r:id="rId6"/>
+    <sheet name="Run" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913" fullCalcOnLoad="1" fullPrecision="1"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Key</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Code_Image_Name</t>
   </si>
   <si>
-    <t>fptuxaes/aes-dotnet8:latest</t>
-  </si>
-  <si>
     <t>Code_Container_Name</t>
   </si>
   <si>
@@ -207,14 +204,22 @@
   </si>
   <si>
     <t>copy_essential_files_and_folders</t>
+  </si>
+  <si>
+    <t>fptuxaes/aes-dotnet8-console:latest</t>
+  </si>
+  <si>
+    <t>generate_connection_file</t>
+  </si>
+  <si>
+    <t>generate_database_script</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -442,85 +447,85 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" applyNumberFormat="0" fontId="5" applyFont="1" fillId="0" applyFill="0" borderId="0" applyBorder="0" applyProtection="0" applyAlignment="0"/>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="3" applyFill="1" borderId="2" applyBorder="1" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="3" applyFill="1" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="3" applyFill="1" borderId="3" applyBorder="1" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="3" applyFill="1" borderId="4" applyBorder="1" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="2" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="4" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="5" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="4" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="3" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="0" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="6" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="7" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" applyFont="1" fillId="4" applyFill="1" borderId="1" applyBorder="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" applyFont="1" fillId="0" borderId="1" applyBorder="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="3" applyFill="1" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="3" applyFill="1" borderId="4" applyBorder="1" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" applyFont="1" fillId="3" applyFill="1" borderId="3" applyBorder="1" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="8" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="8" applyFill="1" borderId="5" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="9" applyFill="1" borderId="6" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" applyFont="1" fillId="9" applyFill="1" borderId="7" applyBorder="1" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" applyFont="1" fillId="10" applyFill="1" borderId="8" applyBorder="1" xfId="0"/>
-    <xf numFmtId="0" fontId="4" applyFont="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -861,14 +866,14 @@
   <dimension ref="A1:B23"/>
   <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.796875" customWidth="1" style="1"/>
-    <col min="2" max="2" width="42.8984375" customWidth="1" style="1"/>
-    <col min="3" max="3" bestFit="1" width="10.59765625" customWidth="1" style="1"/>
-    <col min="4" max="4" width="9.09765625" customWidth="1" style="1"/>
-    <col min="5" max="16384" width="9.09765625" customWidth="1" style="1"/>
+    <col min="1" max="1" width="30.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="42.8984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="9.09765625" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.09765625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -876,7 +881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
@@ -884,7 +889,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1">
+    <row r="3" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>4</v>
       </c>
@@ -892,160 +897,159 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="21.75" customHeight="1">
+    <row r="4" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="s">
+      <c r="B5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="10" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="21" t="s">
+      <c r="B6" s="19">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="22">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="23" t="s">
+      <c r="B7" s="21">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="24">
-        <v>8081</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="s">
+      <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="1" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="s">
+      <c r="B9" s="10"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="10"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="s">
+      <c r="B10" s="11"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="11"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="s">
+      <c r="B11" s="11"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="11"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="s">
+      <c r="B12" s="12"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="12"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="s">
+      <c r="B13" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="13" t="s">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="s">
+      <c r="B14" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="13" t="s">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>22</v>
       </c>
       <c r="B15" s="13">
         <v>1433</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="13">
         <v>1434</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="13" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="s">
+      <c r="B18" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="17" t="s">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="s">
+      <c r="B19" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="14" t="s">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="s">
+      <c r="B20" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="14" t="s">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="s">
+      <c r="B21" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="14" t="s">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="s">
+      <c r="B22" s="13"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
         <v>34</v>
-      </c>
-      <c r="B22" s="13"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="s">
-        <v>35</v>
       </c>
       <c r="B23" s="15"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B18" r:id="rId1"/>
+    <hyperlink ref="B18" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1054,150 +1058,161 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.59765625" customWidth="1" style="6"/>
-    <col min="2" max="2" width="37.19921875" customWidth="1" style="7"/>
+    <col min="1" max="1" width="21.59765625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="37.19921875" style="7" customWidth="1"/>
     <col min="3" max="3" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="18" t="s">
+      <c r="B2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="25"/>
+      <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="18"/>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="25"/>
+      <c r="B4" s="3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="18"/>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="25"/>
+      <c r="B5" s="3" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18"/>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="3" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="25"/>
+      <c r="B6" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18"/>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="4" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="s">
+      <c r="B7" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="25"/>
+      <c r="B8" s="3" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18"/>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="25"/>
+      <c r="B9" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="3"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="18"/>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="25"/>
+      <c r="B10" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="18"/>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="27"/>
+      <c r="B11" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="20"/>
-      <c r="B11" s="4" t="s">
-        <v>56</v>
-      </c>
       <c r="C11" s="4"/>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="2">
     <mergeCell ref="A2:A6"/>
     <mergeCell ref="A7:A11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5A8B865-FC4E-42B9-9CDF-4A31D67503FE}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1" style="25"/>
-    <col min="2" max="2" bestFit="1" width="27.81640625" customWidth="1" style="25"/>
-    <col min="3" max="16384" width="8.90625" customWidth="1" style="25"/>
+    <col min="1" max="1" width="7" style="22" customWidth="1"/>
+    <col min="2" max="2" width="27.796875" style="22" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.8984375" style="22" customWidth="1"/>
+    <col min="4" max="16384" width="8.8984375" style="22"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="26" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="24">
+        <v>1</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="24">
+        <v>2</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="27">
-        <v>1</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="27"/>
-      <c r="B3" s="27"/>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="22">
+        <v>3</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>61</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>